<commit_message>
changement du vto balde
</commit_message>
<xml_diff>
--- a/vto_list.xlsx
+++ b/vto_list.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29629"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Downloads\Dossier LOUMA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="91" documentId="11_62E75E214BEF08387827ABE3F4F2BDEBE23AB00D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{60AF6145-723E-4584-AC1F-01138DCA7977}"/>
+  <xr:revisionPtr revIDLastSave="95" documentId="11_62E75E214BEF08387827ABE3F4F2BDEBE23AB00D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9BEF439B-869A-4A3F-AE9E-B46D81BD02E6}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7050" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -320,13 +320,13 @@
     <t>DR SUD</t>
   </si>
   <si>
+    <t xml:space="preserve">COUMBA </t>
+  </si>
+  <si>
+    <t>pvt_mwadk173</t>
+  </si>
+  <si>
     <t>HAMADOU</t>
-  </si>
-  <si>
-    <t>BALDE</t>
-  </si>
-  <si>
-    <t>pvt_mwadk236</t>
   </si>
   <si>
     <t>MBALLO</t>
@@ -703,22 +703,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
@@ -739,10 +727,22 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1056,10 +1056,10 @@
       </c>
     </row>
     <row r="2" spans="1:6" ht="14.45" customHeight="1">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="B2" s="20" t="s">
         <v>7</v>
       </c>
       <c r="C2" s="2" t="s">
@@ -1076,8 +1076,8 @@
       </c>
     </row>
     <row r="3" spans="1:6" ht="14.45" customHeight="1">
-      <c r="A3" s="13"/>
-      <c r="B3" s="11"/>
+      <c r="A3" s="19"/>
+      <c r="B3" s="21"/>
       <c r="C3" s="2" t="s">
         <v>11</v>
       </c>
@@ -1092,8 +1092,8 @@
       </c>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="13"/>
-      <c r="B4" s="11"/>
+      <c r="A4" s="19"/>
+      <c r="B4" s="21"/>
       <c r="C4" s="2" t="s">
         <v>14</v>
       </c>
@@ -1108,8 +1108,8 @@
       </c>
     </row>
     <row r="5" spans="1:6">
-      <c r="A5" s="13"/>
-      <c r="B5" s="11"/>
+      <c r="A5" s="19"/>
+      <c r="B5" s="21"/>
       <c r="C5" s="9" t="s">
         <v>17</v>
       </c>
@@ -1124,10 +1124,10 @@
       </c>
     </row>
     <row r="6" spans="1:6">
-      <c r="A6" s="22" t="s">
+      <c r="A6" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="23" t="s">
+      <c r="B6" s="10" t="s">
         <v>20</v>
       </c>
       <c r="C6" s="8" t="s">
@@ -1144,8 +1144,8 @@
       </c>
     </row>
     <row r="7" spans="1:6">
-      <c r="A7" s="22"/>
-      <c r="B7" s="23"/>
+      <c r="A7" s="11"/>
+      <c r="B7" s="10"/>
       <c r="C7" s="8" t="s">
         <v>24</v>
       </c>
@@ -1160,8 +1160,8 @@
       </c>
     </row>
     <row r="8" spans="1:6" ht="14.45" customHeight="1">
-      <c r="A8" s="22"/>
-      <c r="B8" s="23"/>
+      <c r="A8" s="11"/>
+      <c r="B8" s="10"/>
       <c r="C8" s="8" t="s">
         <v>27</v>
       </c>
@@ -1176,8 +1176,8 @@
       </c>
     </row>
     <row r="9" spans="1:6" ht="14.45" customHeight="1">
-      <c r="A9" s="22"/>
-      <c r="B9" s="23"/>
+      <c r="A9" s="11"/>
+      <c r="B9" s="10"/>
       <c r="C9" s="8" t="s">
         <v>30</v>
       </c>
@@ -1192,10 +1192,10 @@
       </c>
     </row>
     <row r="10" spans="1:6">
-      <c r="A10" s="12" t="s">
+      <c r="A10" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="21" t="s">
         <v>34</v>
       </c>
       <c r="C10" s="2" t="s">
@@ -1212,8 +1212,8 @@
       </c>
     </row>
     <row r="11" spans="1:6">
-      <c r="A11" s="13"/>
-      <c r="B11" s="11" t="s">
+      <c r="A11" s="19"/>
+      <c r="B11" s="21" t="s">
         <v>34</v>
       </c>
       <c r="C11" s="2" t="s">
@@ -1230,8 +1230,8 @@
       </c>
     </row>
     <row r="12" spans="1:6">
-      <c r="A12" s="13"/>
-      <c r="B12" s="11" t="s">
+      <c r="A12" s="19"/>
+      <c r="B12" s="21" t="s">
         <v>34</v>
       </c>
       <c r="C12" s="2" t="s">
@@ -1248,8 +1248,8 @@
       </c>
     </row>
     <row r="13" spans="1:6">
-      <c r="A13" s="14"/>
-      <c r="B13" s="15" t="s">
+      <c r="A13" s="22"/>
+      <c r="B13" s="23" t="s">
         <v>34</v>
       </c>
       <c r="C13" s="2" t="s">
@@ -1266,10 +1266,10 @@
       </c>
     </row>
     <row r="14" spans="1:6">
-      <c r="A14" s="12" t="s">
+      <c r="A14" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="20" t="s">
         <v>46</v>
       </c>
       <c r="C14" s="2" t="s">
@@ -1286,8 +1286,8 @@
       </c>
     </row>
     <row r="15" spans="1:6">
-      <c r="A15" s="13"/>
-      <c r="B15" s="11" t="s">
+      <c r="A15" s="19"/>
+      <c r="B15" s="21" t="s">
         <v>46</v>
       </c>
       <c r="C15" s="2" t="s">
@@ -1304,8 +1304,8 @@
       </c>
     </row>
     <row r="16" spans="1:6">
-      <c r="A16" s="13"/>
-      <c r="B16" s="11" t="s">
+      <c r="A16" s="19"/>
+      <c r="B16" s="21" t="s">
         <v>46</v>
       </c>
       <c r="C16" s="2" t="s">
@@ -1322,8 +1322,8 @@
       </c>
     </row>
     <row r="17" spans="1:6">
-      <c r="A17" s="14"/>
-      <c r="B17" s="15" t="s">
+      <c r="A17" s="22"/>
+      <c r="B17" s="23" t="s">
         <v>46</v>
       </c>
       <c r="C17" s="2" t="s">
@@ -1340,10 +1340,10 @@
       </c>
     </row>
     <row r="18" spans="1:6">
-      <c r="A18" s="12" t="s">
+      <c r="A18" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="B18" s="10" t="s">
+      <c r="B18" s="20" t="s">
         <v>60</v>
       </c>
       <c r="C18" s="2" t="s">
@@ -1360,8 +1360,8 @@
       </c>
     </row>
     <row r="19" spans="1:6">
-      <c r="A19" s="13"/>
-      <c r="B19" s="11" t="s">
+      <c r="A19" s="19"/>
+      <c r="B19" s="21" t="s">
         <v>60</v>
       </c>
       <c r="C19" s="2" t="s">
@@ -1378,8 +1378,8 @@
       </c>
     </row>
     <row r="20" spans="1:6">
-      <c r="A20" s="13"/>
-      <c r="B20" s="11" t="s">
+      <c r="A20" s="19"/>
+      <c r="B20" s="21" t="s">
         <v>60</v>
       </c>
       <c r="C20" s="2" t="s">
@@ -1396,8 +1396,8 @@
       </c>
     </row>
     <row r="21" spans="1:6">
-      <c r="A21" s="14"/>
-      <c r="B21" s="15" t="s">
+      <c r="A21" s="22"/>
+      <c r="B21" s="23" t="s">
         <v>60</v>
       </c>
       <c r="C21" s="2" t="s">
@@ -1414,10 +1414,10 @@
       </c>
     </row>
     <row r="22" spans="1:6">
-      <c r="A22" s="12" t="s">
+      <c r="A22" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="B22" s="10" t="s">
+      <c r="B22" s="20" t="s">
         <v>73</v>
       </c>
       <c r="C22" s="2" t="s">
@@ -1434,8 +1434,8 @@
       </c>
     </row>
     <row r="23" spans="1:6">
-      <c r="A23" s="13"/>
-      <c r="B23" s="11" t="s">
+      <c r="A23" s="19"/>
+      <c r="B23" s="21" t="s">
         <v>73</v>
       </c>
       <c r="C23" s="2" t="s">
@@ -1452,8 +1452,8 @@
       </c>
     </row>
     <row r="24" spans="1:6">
-      <c r="A24" s="13"/>
-      <c r="B24" s="11" t="s">
+      <c r="A24" s="19"/>
+      <c r="B24" s="21" t="s">
         <v>73</v>
       </c>
       <c r="C24" s="2" t="s">
@@ -1470,8 +1470,8 @@
       </c>
     </row>
     <row r="25" spans="1:6">
-      <c r="A25" s="14"/>
-      <c r="B25" s="15" t="s">
+      <c r="A25" s="22"/>
+      <c r="B25" s="23" t="s">
         <v>73</v>
       </c>
       <c r="C25" s="2" t="s">
@@ -1488,10 +1488,10 @@
       </c>
     </row>
     <row r="26" spans="1:6">
-      <c r="A26" s="12" t="s">
+      <c r="A26" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="B26" s="10" t="s">
+      <c r="B26" s="20" t="s">
         <v>88</v>
       </c>
       <c r="C26" s="2" t="s">
@@ -1508,34 +1508,34 @@
       </c>
     </row>
     <row r="27" spans="1:6">
-      <c r="A27" s="13" t="s">
+      <c r="A27" s="19" t="s">
         <v>92</v>
       </c>
-      <c r="B27" s="11" t="s">
+      <c r="B27" s="21" t="s">
         <v>88</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>93</v>
       </c>
       <c r="D27" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E27" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="E27" s="2" t="s">
+      <c r="F27" s="2">
+        <v>772105935</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
+      <c r="A28" s="19" t="s">
+        <v>92</v>
+      </c>
+      <c r="B28" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="C28" s="2" t="s">
         <v>95</v>
-      </c>
-      <c r="F27" s="2">
-        <v>778525987</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6">
-      <c r="A28" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="B28" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>93</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>96</v>
@@ -1548,10 +1548,10 @@
       </c>
     </row>
     <row r="29" spans="1:6">
-      <c r="A29" s="14" t="s">
+      <c r="A29" s="22" t="s">
         <v>92</v>
       </c>
-      <c r="B29" s="15" t="s">
+      <c r="B29" s="23" t="s">
         <v>88</v>
       </c>
       <c r="C29" s="2" t="s">
@@ -1568,10 +1568,10 @@
       </c>
     </row>
     <row r="30" spans="1:6">
-      <c r="A30" s="12" t="s">
+      <c r="A30" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="B30" s="10" t="s">
+      <c r="B30" s="20" t="s">
         <v>100</v>
       </c>
       <c r="C30" s="2" t="s">
@@ -1588,10 +1588,10 @@
       </c>
     </row>
     <row r="31" spans="1:6">
-      <c r="A31" s="13" t="s">
+      <c r="A31" s="19" t="s">
         <v>104</v>
       </c>
-      <c r="B31" s="11" t="s">
+      <c r="B31" s="21" t="s">
         <v>100</v>
       </c>
       <c r="C31" s="2" t="s">
@@ -1608,10 +1608,10 @@
       </c>
     </row>
     <row r="32" spans="1:6">
-      <c r="A32" s="13" t="s">
+      <c r="A32" s="19" t="s">
         <v>104</v>
       </c>
-      <c r="B32" s="11" t="s">
+      <c r="B32" s="21" t="s">
         <v>100</v>
       </c>
       <c r="C32" s="2" t="s">
@@ -1628,10 +1628,10 @@
       </c>
     </row>
     <row r="33" spans="1:6">
-      <c r="A33" s="14" t="s">
+      <c r="A33" s="22" t="s">
         <v>104</v>
       </c>
-      <c r="B33" s="15" t="s">
+      <c r="B33" s="23" t="s">
         <v>100</v>
       </c>
       <c r="C33" s="2" t="s">
@@ -1648,10 +1648,10 @@
       </c>
     </row>
     <row r="34" spans="1:6">
-      <c r="A34" s="12" t="s">
+      <c r="A34" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="B34" s="10" t="s">
+      <c r="B34" s="20" t="s">
         <v>113</v>
       </c>
       <c r="C34" s="2" t="s">
@@ -1668,10 +1668,10 @@
       </c>
     </row>
     <row r="35" spans="1:6">
-      <c r="A35" s="13" t="s">
+      <c r="A35" s="19" t="s">
         <v>116</v>
       </c>
-      <c r="B35" s="11" t="s">
+      <c r="B35" s="21" t="s">
         <v>113</v>
       </c>
       <c r="C35" s="2" t="s">
@@ -1688,10 +1688,10 @@
       </c>
     </row>
     <row r="36" spans="1:6">
-      <c r="A36" s="13" t="s">
+      <c r="A36" s="19" t="s">
         <v>116</v>
       </c>
-      <c r="B36" s="11" t="s">
+      <c r="B36" s="21" t="s">
         <v>113</v>
       </c>
       <c r="C36" s="2" t="s">
@@ -1708,10 +1708,10 @@
       </c>
     </row>
     <row r="37" spans="1:6">
-      <c r="A37" s="14" t="s">
+      <c r="A37" s="22" t="s">
         <v>116</v>
       </c>
-      <c r="B37" s="15" t="s">
+      <c r="B37" s="23" t="s">
         <v>113</v>
       </c>
       <c r="C37" s="2" t="s">
@@ -1728,10 +1728,10 @@
       </c>
     </row>
     <row r="38" spans="1:6" ht="14.45" customHeight="1">
-      <c r="A38" s="12" t="s">
+      <c r="A38" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="B38" s="10" t="s">
+      <c r="B38" s="20" t="s">
         <v>124</v>
       </c>
       <c r="C38" s="2" t="s">
@@ -1748,8 +1748,8 @@
       </c>
     </row>
     <row r="39" spans="1:6" ht="14.45" customHeight="1">
-      <c r="A39" s="13"/>
-      <c r="B39" s="11" t="s">
+      <c r="A39" s="19"/>
+      <c r="B39" s="21" t="s">
         <v>124</v>
       </c>
       <c r="C39" s="2" t="s">
@@ -1766,8 +1766,8 @@
       </c>
     </row>
     <row r="40" spans="1:6" ht="14.45" customHeight="1">
-      <c r="A40" s="13"/>
-      <c r="B40" s="11" t="s">
+      <c r="A40" s="19"/>
+      <c r="B40" s="21" t="s">
         <v>124</v>
       </c>
       <c r="C40" s="2" t="s">
@@ -1784,8 +1784,8 @@
       </c>
     </row>
     <row r="41" spans="1:6" ht="14.45" customHeight="1">
-      <c r="A41" s="14"/>
-      <c r="B41" s="15" t="s">
+      <c r="A41" s="22"/>
+      <c r="B41" s="23" t="s">
         <v>124</v>
       </c>
       <c r="C41" s="2" t="s">
@@ -1802,10 +1802,10 @@
       </c>
     </row>
     <row r="42" spans="1:6">
-      <c r="A42" s="12" t="s">
+      <c r="A42" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="B42" s="10" t="s">
+      <c r="B42" s="20" t="s">
         <v>136</v>
       </c>
       <c r="C42" s="2" t="s">
@@ -1822,10 +1822,10 @@
       </c>
     </row>
     <row r="43" spans="1:6">
-      <c r="A43" s="13" t="s">
+      <c r="A43" s="19" t="s">
         <v>92</v>
       </c>
-      <c r="B43" s="11" t="s">
+      <c r="B43" s="21" t="s">
         <v>136</v>
       </c>
       <c r="C43" s="2" t="s">
@@ -1842,10 +1842,10 @@
       </c>
     </row>
     <row r="44" spans="1:6">
-      <c r="A44" s="13" t="s">
+      <c r="A44" s="19" t="s">
         <v>92</v>
       </c>
-      <c r="B44" s="11" t="s">
+      <c r="B44" s="21" t="s">
         <v>136</v>
       </c>
       <c r="C44" s="2" t="s">
@@ -1862,10 +1862,10 @@
       </c>
     </row>
     <row r="45" spans="1:6">
-      <c r="A45" s="14" t="s">
+      <c r="A45" s="22" t="s">
         <v>92</v>
       </c>
-      <c r="B45" s="15" t="s">
+      <c r="B45" s="23" t="s">
         <v>136</v>
       </c>
       <c r="C45" s="2" t="s">
@@ -1885,7 +1885,7 @@
       <c r="A46" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B46" s="10" t="s">
+      <c r="B46" s="20" t="s">
         <v>148</v>
       </c>
       <c r="C46" s="2" t="s">
@@ -1903,7 +1903,7 @@
     </row>
     <row r="47" spans="1:6">
       <c r="A47" s="6"/>
-      <c r="B47" s="11" t="s">
+      <c r="B47" s="21" t="s">
         <v>148</v>
       </c>
       <c r="C47" s="2" t="s">
@@ -1921,7 +1921,7 @@
     </row>
     <row r="48" spans="1:6">
       <c r="A48" s="6"/>
-      <c r="B48" s="11" t="s">
+      <c r="B48" s="21" t="s">
         <v>148</v>
       </c>
       <c r="C48" s="2" t="s">
@@ -1939,7 +1939,7 @@
     </row>
     <row r="49" spans="1:6">
       <c r="A49" s="6"/>
-      <c r="B49" s="11" t="s">
+      <c r="B49" s="21" t="s">
         <v>148</v>
       </c>
       <c r="C49" s="9" t="s">
@@ -1956,10 +1956,10 @@
       </c>
     </row>
     <row r="50" spans="1:6">
-      <c r="A50" s="16" t="s">
+      <c r="A50" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="B50" s="19" t="s">
+      <c r="B50" s="15" t="s">
         <v>20</v>
       </c>
       <c r="C50" s="8" t="s">
@@ -1976,8 +1976,8 @@
       </c>
     </row>
     <row r="51" spans="1:6">
-      <c r="A51" s="17"/>
-      <c r="B51" s="20"/>
+      <c r="A51" s="13"/>
+      <c r="B51" s="16"/>
       <c r="C51" s="8" t="s">
         <v>24</v>
       </c>
@@ -1992,8 +1992,8 @@
       </c>
     </row>
     <row r="52" spans="1:6">
-      <c r="A52" s="17"/>
-      <c r="B52" s="20"/>
+      <c r="A52" s="13"/>
+      <c r="B52" s="16"/>
       <c r="C52" s="8" t="s">
         <v>27</v>
       </c>
@@ -2008,8 +2008,8 @@
       </c>
     </row>
     <row r="53" spans="1:6">
-      <c r="A53" s="18"/>
-      <c r="B53" s="21"/>
+      <c r="A53" s="14"/>
+      <c r="B53" s="17"/>
       <c r="C53" s="8" t="s">
         <v>30</v>
       </c>
@@ -2026,6 +2026,15 @@
   </sheetData>
   <autoFilter ref="A1:F49" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="25">
+    <mergeCell ref="A42:A45"/>
+    <mergeCell ref="B42:B45"/>
+    <mergeCell ref="B46:B49"/>
+    <mergeCell ref="A30:A33"/>
+    <mergeCell ref="B30:B33"/>
+    <mergeCell ref="A34:A37"/>
+    <mergeCell ref="B34:B37"/>
+    <mergeCell ref="A38:A41"/>
+    <mergeCell ref="B38:B41"/>
     <mergeCell ref="B6:B9"/>
     <mergeCell ref="A6:A9"/>
     <mergeCell ref="A50:A53"/>
@@ -2042,15 +2051,6 @@
     <mergeCell ref="B22:B25"/>
     <mergeCell ref="A26:A29"/>
     <mergeCell ref="B26:B29"/>
-    <mergeCell ref="A42:A45"/>
-    <mergeCell ref="B42:B45"/>
-    <mergeCell ref="B46:B49"/>
-    <mergeCell ref="A30:A33"/>
-    <mergeCell ref="B30:B33"/>
-    <mergeCell ref="A34:A37"/>
-    <mergeCell ref="B34:B37"/>
-    <mergeCell ref="A38:A41"/>
-    <mergeCell ref="B38:B41"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
ajout du vto balde jusqu'au payement
</commit_message>
<xml_diff>
--- a/vto_list.xlsx
+++ b/vto_list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Downloads\Dossier LOUMA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="95" documentId="11_62E75E214BEF08387827ABE3F4F2BDEBE23AB00D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9BEF439B-869A-4A3F-AE9E-B46D81BD02E6}"/>
+  <xr:revisionPtr revIDLastSave="109" documentId="11_62E75E214BEF08387827ABE3F4F2BDEBE23AB00D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8C35196B-F670-4F5B-B177-60A4FEC348B6}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7050" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Liste VTO" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Liste VTO'!$A$1:$F$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Liste VTO'!$A$1:$F$50</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="162">
   <si>
     <t>DRV</t>
   </si>
@@ -317,6 +317,15 @@
     <t>pvt_mwadk0290</t>
   </si>
   <si>
+    <t>HAMADOU</t>
+  </si>
+  <si>
+    <t>BALDE</t>
+  </si>
+  <si>
+    <t>pvt_mwadk236</t>
+  </si>
+  <si>
     <t>DR SUD</t>
   </si>
   <si>
@@ -324,9 +333,6 @@
   </si>
   <si>
     <t>pvt_mwadk173</t>
-  </si>
-  <si>
-    <t>HAMADOU</t>
   </si>
   <si>
     <t>MBALLO</t>
@@ -703,6 +709,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -726,24 +750,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1025,7 +1031,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:F54"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="58.85546875" bestFit="1" customWidth="1"/>
@@ -1056,10 +1062,10 @@
       </c>
     </row>
     <row r="2" spans="1:6" ht="14.45" customHeight="1">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="20" t="s">
+      <c r="B2" s="13" t="s">
         <v>7</v>
       </c>
       <c r="C2" s="2" t="s">
@@ -1076,8 +1082,8 @@
       </c>
     </row>
     <row r="3" spans="1:6" ht="14.45" customHeight="1">
-      <c r="A3" s="19"/>
-      <c r="B3" s="21"/>
+      <c r="A3" s="11"/>
+      <c r="B3" s="14"/>
       <c r="C3" s="2" t="s">
         <v>11</v>
       </c>
@@ -1092,8 +1098,8 @@
       </c>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="19"/>
-      <c r="B4" s="21"/>
+      <c r="A4" s="11"/>
+      <c r="B4" s="14"/>
       <c r="C4" s="2" t="s">
         <v>14</v>
       </c>
@@ -1108,8 +1114,8 @@
       </c>
     </row>
     <row r="5" spans="1:6">
-      <c r="A5" s="19"/>
-      <c r="B5" s="21"/>
+      <c r="A5" s="11"/>
+      <c r="B5" s="14"/>
       <c r="C5" s="9" t="s">
         <v>17</v>
       </c>
@@ -1124,10 +1130,10 @@
       </c>
     </row>
     <row r="6" spans="1:6">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="16" t="s">
         <v>20</v>
       </c>
       <c r="C6" s="8" t="s">
@@ -1144,8 +1150,8 @@
       </c>
     </row>
     <row r="7" spans="1:6">
-      <c r="A7" s="11"/>
-      <c r="B7" s="10"/>
+      <c r="A7" s="17"/>
+      <c r="B7" s="16"/>
       <c r="C7" s="8" t="s">
         <v>24</v>
       </c>
@@ -1160,8 +1166,8 @@
       </c>
     </row>
     <row r="8" spans="1:6" ht="14.45" customHeight="1">
-      <c r="A8" s="11"/>
-      <c r="B8" s="10"/>
+      <c r="A8" s="17"/>
+      <c r="B8" s="16"/>
       <c r="C8" s="8" t="s">
         <v>27</v>
       </c>
@@ -1176,8 +1182,8 @@
       </c>
     </row>
     <row r="9" spans="1:6" ht="14.45" customHeight="1">
-      <c r="A9" s="11"/>
-      <c r="B9" s="10"/>
+      <c r="A9" s="17"/>
+      <c r="B9" s="16"/>
       <c r="C9" s="8" t="s">
         <v>30</v>
       </c>
@@ -1192,10 +1198,10 @@
       </c>
     </row>
     <row r="10" spans="1:6">
-      <c r="A10" s="18" t="s">
+      <c r="A10" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="B10" s="21" t="s">
+      <c r="B10" s="14" t="s">
         <v>34</v>
       </c>
       <c r="C10" s="2" t="s">
@@ -1212,8 +1218,8 @@
       </c>
     </row>
     <row r="11" spans="1:6">
-      <c r="A11" s="19"/>
-      <c r="B11" s="21" t="s">
+      <c r="A11" s="11"/>
+      <c r="B11" s="14" t="s">
         <v>34</v>
       </c>
       <c r="C11" s="2" t="s">
@@ -1230,8 +1236,8 @@
       </c>
     </row>
     <row r="12" spans="1:6">
-      <c r="A12" s="19"/>
-      <c r="B12" s="21" t="s">
+      <c r="A12" s="11"/>
+      <c r="B12" s="14" t="s">
         <v>34</v>
       </c>
       <c r="C12" s="2" t="s">
@@ -1248,8 +1254,8 @@
       </c>
     </row>
     <row r="13" spans="1:6">
-      <c r="A13" s="22"/>
-      <c r="B13" s="23" t="s">
+      <c r="A13" s="12"/>
+      <c r="B13" s="15" t="s">
         <v>34</v>
       </c>
       <c r="C13" s="2" t="s">
@@ -1266,10 +1272,10 @@
       </c>
     </row>
     <row r="14" spans="1:6">
-      <c r="A14" s="18" t="s">
+      <c r="A14" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="B14" s="20" t="s">
+      <c r="B14" s="13" t="s">
         <v>46</v>
       </c>
       <c r="C14" s="2" t="s">
@@ -1286,8 +1292,8 @@
       </c>
     </row>
     <row r="15" spans="1:6">
-      <c r="A15" s="19"/>
-      <c r="B15" s="21" t="s">
+      <c r="A15" s="11"/>
+      <c r="B15" s="14" t="s">
         <v>46</v>
       </c>
       <c r="C15" s="2" t="s">
@@ -1304,8 +1310,8 @@
       </c>
     </row>
     <row r="16" spans="1:6">
-      <c r="A16" s="19"/>
-      <c r="B16" s="21" t="s">
+      <c r="A16" s="11"/>
+      <c r="B16" s="14" t="s">
         <v>46</v>
       </c>
       <c r="C16" s="2" t="s">
@@ -1322,8 +1328,8 @@
       </c>
     </row>
     <row r="17" spans="1:6">
-      <c r="A17" s="22"/>
-      <c r="B17" s="23" t="s">
+      <c r="A17" s="12"/>
+      <c r="B17" s="15" t="s">
         <v>46</v>
       </c>
       <c r="C17" s="2" t="s">
@@ -1340,10 +1346,10 @@
       </c>
     </row>
     <row r="18" spans="1:6">
-      <c r="A18" s="18" t="s">
+      <c r="A18" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="B18" s="20" t="s">
+      <c r="B18" s="13" t="s">
         <v>60</v>
       </c>
       <c r="C18" s="2" t="s">
@@ -1360,8 +1366,8 @@
       </c>
     </row>
     <row r="19" spans="1:6">
-      <c r="A19" s="19"/>
-      <c r="B19" s="21" t="s">
+      <c r="A19" s="11"/>
+      <c r="B19" s="14" t="s">
         <v>60</v>
       </c>
       <c r="C19" s="2" t="s">
@@ -1378,8 +1384,8 @@
       </c>
     </row>
     <row r="20" spans="1:6">
-      <c r="A20" s="19"/>
-      <c r="B20" s="21" t="s">
+      <c r="A20" s="11"/>
+      <c r="B20" s="14" t="s">
         <v>60</v>
       </c>
       <c r="C20" s="2" t="s">
@@ -1396,8 +1402,8 @@
       </c>
     </row>
     <row r="21" spans="1:6">
-      <c r="A21" s="22"/>
-      <c r="B21" s="23" t="s">
+      <c r="A21" s="12"/>
+      <c r="B21" s="15" t="s">
         <v>60</v>
       </c>
       <c r="C21" s="2" t="s">
@@ -1414,10 +1420,10 @@
       </c>
     </row>
     <row r="22" spans="1:6">
-      <c r="A22" s="18" t="s">
+      <c r="A22" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="B22" s="20" t="s">
+      <c r="B22" s="13" t="s">
         <v>73</v>
       </c>
       <c r="C22" s="2" t="s">
@@ -1434,8 +1440,8 @@
       </c>
     </row>
     <row r="23" spans="1:6">
-      <c r="A23" s="19"/>
-      <c r="B23" s="21" t="s">
+      <c r="A23" s="11"/>
+      <c r="B23" s="14" t="s">
         <v>73</v>
       </c>
       <c r="C23" s="2" t="s">
@@ -1452,8 +1458,8 @@
       </c>
     </row>
     <row r="24" spans="1:6">
-      <c r="A24" s="19"/>
-      <c r="B24" s="21" t="s">
+      <c r="A24" s="11"/>
+      <c r="B24" s="14" t="s">
         <v>73</v>
       </c>
       <c r="C24" s="2" t="s">
@@ -1470,8 +1476,8 @@
       </c>
     </row>
     <row r="25" spans="1:6">
-      <c r="A25" s="22"/>
-      <c r="B25" s="23" t="s">
+      <c r="A25" s="12"/>
+      <c r="B25" s="15" t="s">
         <v>73</v>
       </c>
       <c r="C25" s="2" t="s">
@@ -1488,10 +1494,10 @@
       </c>
     </row>
     <row r="26" spans="1:6">
-      <c r="A26" s="18" t="s">
+      <c r="A26" s="10" t="s">
         <v>87</v>
       </c>
-      <c r="B26" s="20" t="s">
+      <c r="B26" s="13" t="s">
         <v>88</v>
       </c>
       <c r="C26" s="2" t="s">
@@ -1508,537 +1514,542 @@
       </c>
     </row>
     <row r="27" spans="1:6">
-      <c r="A27" s="19" t="s">
+      <c r="A27" s="11"/>
+      <c r="B27" s="14"/>
+      <c r="C27" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="B27" s="21" t="s">
-        <v>88</v>
-      </c>
-      <c r="C27" s="2" t="s">
+      <c r="D27" s="2" t="s">
         <v>93</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>31</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="F27" s="2">
-        <v>772105935</v>
-      </c>
+      <c r="F27" s="2"/>
     </row>
     <row r="28" spans="1:6">
-      <c r="A28" s="19" t="s">
-        <v>92</v>
-      </c>
-      <c r="B28" s="21" t="s">
+      <c r="A28" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="B28" s="14" t="s">
         <v>88</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>96</v>
+        <v>31</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>97</v>
       </c>
       <c r="F28" s="2">
-        <v>772104981</v>
+        <v>772105935</v>
       </c>
     </row>
     <row r="29" spans="1:6">
-      <c r="A29" s="22" t="s">
+      <c r="A29" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="B29" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="C29" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="B29" s="23" t="s">
-        <v>88</v>
-      </c>
-      <c r="C29" s="2" t="s">
+      <c r="D29" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>85</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>99</v>
       </c>
       <c r="F29" s="2">
+        <v>772104981</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6">
+      <c r="A30" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="B30" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="F30" s="2">
         <v>772107591</v>
       </c>
     </row>
-    <row r="30" spans="1:6">
-      <c r="A30" s="18" t="s">
+    <row r="31" spans="1:6">
+      <c r="A31" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="B30" s="20" t="s">
-        <v>100</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="D30" s="2" t="s">
+      <c r="B31" s="13" t="s">
         <v>102</v>
       </c>
-      <c r="E30" s="2" t="s">
+      <c r="C31" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="F30" s="2">
+      <c r="D31" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="F31" s="2">
         <v>777410048</v>
       </c>
     </row>
-    <row r="31" spans="1:6">
-      <c r="A31" s="19" t="s">
-        <v>104</v>
-      </c>
-      <c r="B31" s="21" t="s">
-        <v>100</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="E31" s="2" t="s">
+    <row r="32" spans="1:6">
+      <c r="A32" s="11" t="s">
         <v>106</v>
       </c>
-      <c r="F31" s="2">
-        <v>787656877</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6">
-      <c r="A32" s="19" t="s">
-        <v>104</v>
-      </c>
-      <c r="B32" s="21" t="s">
-        <v>100</v>
+      <c r="B32" s="14" t="s">
+        <v>102</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>107</v>
       </c>
       <c r="D32" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E32" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="E32" s="2" t="s">
+      <c r="F32" s="2">
+        <v>787656877</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6">
+      <c r="A33" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="B33" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="C33" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="F32" s="2">
+      <c r="D33" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="F33" s="2">
         <v>776019823</v>
       </c>
     </row>
-    <row r="33" spans="1:6">
-      <c r="A33" s="22" t="s">
-        <v>104</v>
-      </c>
-      <c r="B33" s="23" t="s">
-        <v>100</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="E33" s="2" t="s">
+    <row r="34" spans="1:6">
+      <c r="A34" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="B34" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="C34" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="F33" s="2">
+      <c r="D34" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="F34" s="2">
         <v>782981141</v>
       </c>
     </row>
-    <row r="34" spans="1:6">
-      <c r="A34" s="18" t="s">
+    <row r="35" spans="1:6">
+      <c r="A35" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="B34" s="20" t="s">
-        <v>113</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="D34" s="2" t="s">
+      <c r="B35" s="13" t="s">
+        <v>115</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="D35" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="E34" s="2" t="s">
+      <c r="E35" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="F35" s="2">
+        <v>788255458</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6">
+      <c r="A36" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="B36" s="14" t="s">
         <v>115</v>
-      </c>
-      <c r="F34" s="2">
-        <v>788255458</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6">
-      <c r="A35" s="19" t="s">
-        <v>116</v>
-      </c>
-      <c r="B35" s="21" t="s">
-        <v>113</v>
-      </c>
-      <c r="C35" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="D35" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="E35" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="F35" s="2">
-        <v>789166919</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6">
-      <c r="A36" s="19" t="s">
-        <v>116</v>
-      </c>
-      <c r="B36" s="21" t="s">
-        <v>113</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>119</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>25</v>
+        <v>85</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>120</v>
       </c>
       <c r="F36" s="2">
-        <v>789151415</v>
+        <v>789166919</v>
       </c>
     </row>
     <row r="37" spans="1:6">
-      <c r="A37" s="22" t="s">
-        <v>116</v>
-      </c>
-      <c r="B37" s="23" t="s">
-        <v>113</v>
+      <c r="A37" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="B37" s="14" t="s">
+        <v>115</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>121</v>
       </c>
       <c r="D37" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E37" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="E37" s="2" t="s">
+      <c r="F37" s="2">
+        <v>789151415</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6">
+      <c r="A38" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="B38" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="C38" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="F37" s="2">
+      <c r="D38" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="F38" s="2">
         <v>789166998</v>
       </c>
     </row>
-    <row r="38" spans="1:6" ht="14.45" customHeight="1">
-      <c r="A38" s="18" t="s">
+    <row r="39" spans="1:6" ht="14.45" customHeight="1">
+      <c r="A39" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="B38" s="20" t="s">
-        <v>124</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="D38" s="2" t="s">
+      <c r="B39" s="13" t="s">
         <v>126</v>
       </c>
-      <c r="E38" s="2" t="s">
+      <c r="C39" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="F38" s="2">
+      <c r="D39" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="F39" s="2">
         <v>781180310</v>
       </c>
     </row>
-    <row r="39" spans="1:6" ht="14.45" customHeight="1">
-      <c r="A39" s="19"/>
-      <c r="B39" s="21" t="s">
-        <v>124</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="E39" s="2" t="s">
+    <row r="40" spans="1:6" ht="14.45" customHeight="1">
+      <c r="A40" s="11"/>
+      <c r="B40" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="C40" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="F39" s="2">
+      <c r="D40" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="F40" s="2">
         <v>781180552</v>
       </c>
     </row>
-    <row r="40" spans="1:6" ht="14.45" customHeight="1">
-      <c r="A40" s="19"/>
-      <c r="B40" s="21" t="s">
-        <v>124</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="E40" s="2" t="s">
+    <row r="41" spans="1:6" ht="14.45" customHeight="1">
+      <c r="A41" s="11"/>
+      <c r="B41" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="C41" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="F40" s="2">
-        <v>787080588</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" ht="14.45" customHeight="1">
-      <c r="A41" s="22"/>
-      <c r="B41" s="23" t="s">
-        <v>124</v>
-      </c>
-      <c r="C41" s="2" t="s">
+      <c r="D41" s="2" t="s">
         <v>134</v>
-      </c>
-      <c r="D41" s="2" t="s">
-        <v>62</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>135</v>
       </c>
       <c r="F41" s="2">
+        <v>787080588</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" ht="14.45" customHeight="1">
+      <c r="A42" s="12"/>
+      <c r="B42" s="15" t="s">
+        <v>126</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="F42" s="2">
         <v>789150406</v>
       </c>
     </row>
-    <row r="42" spans="1:6">
-      <c r="A42" s="18" t="s">
+    <row r="43" spans="1:6">
+      <c r="A43" s="10" t="s">
         <v>87</v>
       </c>
-      <c r="B42" s="20" t="s">
-        <v>136</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="D42" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="E42" s="2" t="s">
+      <c r="B43" s="13" t="s">
         <v>138</v>
-      </c>
-      <c r="F42" s="2">
-        <v>771545210</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6">
-      <c r="A43" s="19" t="s">
-        <v>92</v>
-      </c>
-      <c r="B43" s="21" t="s">
-        <v>136</v>
       </c>
       <c r="C43" s="2" t="s">
         <v>139</v>
       </c>
       <c r="D43" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E43" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="E43" s="2" t="s">
+      <c r="F43" s="2">
+        <v>771545210</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6">
+      <c r="A44" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="B44" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="C44" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="F43" s="2">
+      <c r="D44" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="F44" s="2">
         <v>773958904</v>
       </c>
     </row>
-    <row r="44" spans="1:6">
-      <c r="A44" s="19" t="s">
-        <v>92</v>
-      </c>
-      <c r="B44" s="21" t="s">
-        <v>136</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="D44" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="E44" s="2" t="s">
+    <row r="45" spans="1:6">
+      <c r="A45" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="B45" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="C45" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="F44" s="2">
+      <c r="D45" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="F45" s="2">
         <v>776950987</v>
       </c>
     </row>
-    <row r="45" spans="1:6">
-      <c r="A45" s="22" t="s">
-        <v>92</v>
-      </c>
-      <c r="B45" s="23" t="s">
-        <v>136</v>
-      </c>
-      <c r="C45" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="D45" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="E45" s="2" t="s">
+    <row r="46" spans="1:6">
+      <c r="A46" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="B46" s="15" t="s">
+        <v>138</v>
+      </c>
+      <c r="C46" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="F45" s="2">
+      <c r="D46" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="F46" s="2">
         <v>781825193</v>
       </c>
     </row>
-    <row r="46" spans="1:6">
-      <c r="A46" s="5" t="s">
+    <row r="47" spans="1:6">
+      <c r="A47" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B46" s="20" t="s">
-        <v>148</v>
-      </c>
-      <c r="C46" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="D46" s="2" t="s">
+      <c r="B47" s="13" t="s">
         <v>150</v>
       </c>
-      <c r="E46" s="2" t="s">
+      <c r="C47" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="F46" s="2">
+      <c r="D47" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="E47" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="F47" s="2">
         <v>786180521</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6">
-      <c r="A47" s="6"/>
-      <c r="B47" s="21" t="s">
-        <v>148</v>
-      </c>
-      <c r="C47" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="D47" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="E47" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="F47" s="2">
-        <v>786183517</v>
       </c>
     </row>
     <row r="48" spans="1:6">
       <c r="A48" s="6"/>
-      <c r="B48" s="21" t="s">
-        <v>148</v>
+      <c r="B48" s="14" t="s">
+        <v>150</v>
       </c>
       <c r="C48" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="D48" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="D48" s="2" t="s">
+      <c r="E48" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="E48" s="2" t="s">
-        <v>157</v>
-      </c>
       <c r="F48" s="2">
-        <v>772118585</v>
+        <v>786183517</v>
       </c>
     </row>
     <row r="49" spans="1:6">
       <c r="A49" s="6"/>
-      <c r="B49" s="21" t="s">
-        <v>148</v>
-      </c>
-      <c r="C49" s="9" t="s">
+      <c r="B49" s="14" t="s">
+        <v>150</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="E49" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="F49" s="2">
+        <v>772118585</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6">
+      <c r="A50" s="6"/>
+      <c r="B50" s="14" t="s">
+        <v>150</v>
+      </c>
+      <c r="C50" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="D49" s="9" t="s">
-        <v>158</v>
-      </c>
-      <c r="E49" s="9" t="s">
-        <v>159</v>
-      </c>
-      <c r="F49" s="9">
+      <c r="D50" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="E50" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="F50" s="9">
         <v>787389275</v>
       </c>
     </row>
-    <row r="50" spans="1:6">
-      <c r="A50" s="12" t="s">
+    <row r="51" spans="1:6">
+      <c r="A51" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="B50" s="15" t="s">
+      <c r="B51" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="C50" s="8" t="s">
+      <c r="C51" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="D50" s="7" t="s">
+      <c r="D51" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="E50" s="8" t="s">
+      <c r="E51" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="F50" s="8">
+      <c r="F51" s="8">
         <v>785249423</v>
       </c>
     </row>
-    <row r="51" spans="1:6">
-      <c r="A51" s="13"/>
-      <c r="B51" s="16"/>
-      <c r="C51" s="8" t="s">
+    <row r="52" spans="1:6">
+      <c r="A52" s="19"/>
+      <c r="B52" s="22"/>
+      <c r="C52" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="D51" s="7" t="s">
+      <c r="D52" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="E51" s="8" t="s">
+      <c r="E52" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="F51" s="8">
+      <c r="F52" s="8">
         <v>784720703</v>
       </c>
     </row>
-    <row r="52" spans="1:6">
-      <c r="A52" s="13"/>
-      <c r="B52" s="16"/>
-      <c r="C52" s="8" t="s">
+    <row r="53" spans="1:6">
+      <c r="A53" s="19"/>
+      <c r="B53" s="22"/>
+      <c r="C53" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D52" s="8" t="s">
+      <c r="D53" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="E52" s="8" t="s">
+      <c r="E53" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="F52" s="8">
+      <c r="F53" s="8">
         <v>787979910</v>
       </c>
     </row>
-    <row r="53" spans="1:6">
-      <c r="A53" s="14"/>
-      <c r="B53" s="17"/>
-      <c r="C53" s="8" t="s">
+    <row r="54" spans="1:6">
+      <c r="A54" s="20"/>
+      <c r="B54" s="23"/>
+      <c r="C54" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="D53" s="8" t="s">
+      <c r="D54" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="E53" s="8" t="s">
+      <c r="E54" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="F53" s="8">
+      <c r="F54" s="8">
         <v>789514893</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F49" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:F50" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="25">
-    <mergeCell ref="A42:A45"/>
-    <mergeCell ref="B42:B45"/>
-    <mergeCell ref="B46:B49"/>
-    <mergeCell ref="A30:A33"/>
-    <mergeCell ref="B30:B33"/>
-    <mergeCell ref="A34:A37"/>
-    <mergeCell ref="B34:B37"/>
-    <mergeCell ref="A38:A41"/>
-    <mergeCell ref="B38:B41"/>
     <mergeCell ref="B6:B9"/>
     <mergeCell ref="A6:A9"/>
-    <mergeCell ref="A50:A53"/>
-    <mergeCell ref="B50:B53"/>
+    <mergeCell ref="A51:A54"/>
+    <mergeCell ref="B51:B54"/>
     <mergeCell ref="A2:A5"/>
     <mergeCell ref="B2:B5"/>
     <mergeCell ref="A10:A13"/>
@@ -2049,8 +2060,17 @@
     <mergeCell ref="B18:B21"/>
     <mergeCell ref="A22:A25"/>
     <mergeCell ref="B22:B25"/>
-    <mergeCell ref="A26:A29"/>
-    <mergeCell ref="B26:B29"/>
+    <mergeCell ref="A26:A30"/>
+    <mergeCell ref="B26:B30"/>
+    <mergeCell ref="A43:A46"/>
+    <mergeCell ref="B43:B46"/>
+    <mergeCell ref="B47:B50"/>
+    <mergeCell ref="A31:A34"/>
+    <mergeCell ref="B31:B34"/>
+    <mergeCell ref="A35:A38"/>
+    <mergeCell ref="B35:B38"/>
+    <mergeCell ref="A39:A42"/>
+    <mergeCell ref="B39:B42"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>